<commit_message>
refactor: consolidar 13 funciones en 4 para plan Hobby
</commit_message>
<xml_diff>
--- a/config/maestro-appcontrol.xlsx
+++ b/config/maestro-appcontrol.xlsx
@@ -4,15 +4,16 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="LEEME" sheetId="1" r:id="rId1"/>
-    <sheet name="PROYECTOS" sheetId="2" r:id="rId2"/>
-    <sheet name="USUARIOS" sheetId="3" r:id="rId3"/>
-    <sheet name="CAPITULOS" sheetId="4" r:id="rId4"/>
-    <sheet name="ACTIVIDADES" sheetId="5" r:id="rId5"/>
-    <sheet name="CONTRATISTAS" sheetId="6" r:id="rId6"/>
-    <sheet name="NIVELES" sheetId="7" r:id="rId7"/>
-    <sheet name="UNIDADES" sheetId="8" r:id="rId8"/>
-    <sheet name="CONFIGURACION" sheetId="9" r:id="rId9"/>
-    <sheet name="REGISTRO" sheetId="10" r:id="rId10"/>
+    <sheet name="EMPRESAS" sheetId="2" r:id="rId2"/>
+    <sheet name="PROYECTOS" sheetId="3" r:id="rId3"/>
+    <sheet name="USUARIOS" sheetId="4" r:id="rId4"/>
+    <sheet name="CAPITULOS" sheetId="5" r:id="rId5"/>
+    <sheet name="ACTIVIDADES" sheetId="6" r:id="rId6"/>
+    <sheet name="CONTRATISTAS" sheetId="7" r:id="rId7"/>
+    <sheet name="NIVELES" sheetId="8" r:id="rId8"/>
+    <sheet name="UNIDADES" sheetId="9" r:id="rId9"/>
+    <sheet name="CONFIGURACION" sheetId="10" r:id="rId10"/>
+    <sheet name="REGISTRO" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -406,31 +407,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MAESTRO APPCONTROL - HOJA DE TRABAJO</v>
+        <v>MAESTRO APPCONTROL</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1) Sube este archivo a Google Drive y abrelo con Google Sheets.</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2) Comparte la hoja con la service account (correo en GOOGLE_SERVICE_ACCOUNT_JSON) como EDITOR.</v>
+        <v>CONTIENE DOS PROYECTOS:</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3) Copia el ID de la hoja (entre /d/ y /edit) y pegalo en Vercel: SPREADSHEET_ID.</v>
+        <v xml:space="preserve">  P000 - SALGUERO ELITE 1 (DEMO, con datos de ejemplo)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>4) Redeploy en Vercel y corre: node scripts/smoke.mjs &lt;url&gt; 999000111 1234</v>
+        <v xml:space="preserve">  P001 - SALGUERO ELITE 2 (PRODUCCION, vacio para que tu lo llenes)</v>
       </c>
     </row>
     <row r="6">
@@ -440,28 +441,755 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>REGLA DE ORO: HABILITADO = APLICA SI + ACTIVO SI + CONTRATISTA distinto de 'Sin asignar'.</v>
+        <v>Pasos:</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Solo las filas HABILITADO=SI aparecen en el Grid del residente.</v>
+        <v>1) Sube este archivo a Google Drive y abrelo con Google Sheets.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>REGISTRO es historico: nunca borrar filas; el ultimo estado por unidad es el que manda.</v>
+        <v>2) Comparte la hoja con la service account como EDITOR.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>3) Copia el ID de la hoja (entre /d/ y /edit) a Vercel: SPREADSHEET_ID.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>4) En Vercel: Deployments -&gt; Redeploy.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>5) Abre la app y ejecuta en consola: fetch('/api/seed',{method:'POST'}).then(r=&gt;r.json()).then(console.log)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>6) Entra a /login.html y elige proyecto SALGUERO ELITE 1 para ver la demo.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>CREDENCIALES DEMO:</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v xml:space="preserve">  ADMIN: director@urbanizadorajimenez.com / 123456</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v xml:space="preserve">  RESIDENTE: residente@urbanizadorajimenez.com / 123456</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">  GERENCIA: gerencia@urbanizadorajimenez.com / 123456</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>REGLA DE ORO: HABILITADO = APLICA SI + ACTIVO SI + CONTRATISTA asignado.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Solo las filas HABILITADO=SI aparecen en el Grid del residente.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M16"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PROYECTO</v>
+      </c>
+      <c r="B1" t="str">
+        <v>TORRE</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ACTIVIDAD</v>
+      </c>
+      <c r="D1" t="str">
+        <v>CAPITULO</v>
+      </c>
+      <c r="E1" t="str">
+        <v>NIVEL</v>
+      </c>
+      <c r="F1" t="str">
+        <v>UNIDAD</v>
+      </c>
+      <c r="G1" t="str">
+        <v>APLICA</v>
+      </c>
+      <c r="H1" t="str">
+        <v>ACTIVO</v>
+      </c>
+      <c r="I1" t="str">
+        <v>CONTRATISTA</v>
+      </c>
+      <c r="J1" t="str">
+        <v>HABILITADO</v>
+      </c>
+      <c r="K1" t="str">
+        <v>FECHA_ACTIVACION</v>
+      </c>
+      <c r="L1" t="str">
+        <v>FECHA_DESACTIVACION</v>
+      </c>
+      <c r="M1" t="str">
+        <v>OBSERVACION</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B2" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D2" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E2" t="str">
+        <v>4</v>
+      </c>
+      <c r="F2" t="str">
+        <v>401</v>
+      </c>
+      <c r="G2" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H2" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I2" t="str">
+        <v>CT01</v>
+      </c>
+      <c r="J2" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B3" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D3" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E3" t="str">
+        <v>4</v>
+      </c>
+      <c r="F3" t="str">
+        <v>402</v>
+      </c>
+      <c r="G3" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H3" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Sin asignar</v>
+      </c>
+      <c r="J3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>Falta asignar contratista</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B4" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D4" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E4" t="str">
+        <v>4</v>
+      </c>
+      <c r="F4" t="str">
+        <v>403</v>
+      </c>
+      <c r="G4" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="I4" t="str">
+        <v>CT01</v>
+      </c>
+      <c r="J4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>Pausado</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B5" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D5" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E5" t="str">
+        <v>4</v>
+      </c>
+      <c r="F5" t="str">
+        <v>404</v>
+      </c>
+      <c r="G5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="H5" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I5" t="str">
+        <v>CT01</v>
+      </c>
+      <c r="J5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>No aplica</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B6" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C6" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D6" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E6" t="str">
+        <v>5</v>
+      </c>
+      <c r="F6" t="str">
+        <v>501</v>
+      </c>
+      <c r="G6" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H6" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I6" t="str">
+        <v>CT01</v>
+      </c>
+      <c r="J6" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B7" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ACT010</v>
+      </c>
+      <c r="D7" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5</v>
+      </c>
+      <c r="F7" t="str">
+        <v>502</v>
+      </c>
+      <c r="G7" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H7" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I7" t="str">
+        <v>CT01</v>
+      </c>
+      <c r="J7" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B8" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C8" t="str">
+        <v>ACT020</v>
+      </c>
+      <c r="D8" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="E8" t="str">
+        <v>4</v>
+      </c>
+      <c r="F8" t="str">
+        <v>401</v>
+      </c>
+      <c r="G8" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H8" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I8" t="str">
+        <v>CT02</v>
+      </c>
+      <c r="J8" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B9" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C9" t="str">
+        <v>ACT020</v>
+      </c>
+      <c r="D9" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="E9" t="str">
+        <v>4</v>
+      </c>
+      <c r="F9" t="str">
+        <v>402</v>
+      </c>
+      <c r="G9" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H9" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I9" t="str">
+        <v>CT02</v>
+      </c>
+      <c r="J9" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B10" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ACT020</v>
+      </c>
+      <c r="D10" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="E10" t="str">
+        <v>22</v>
+      </c>
+      <c r="F10" t="str">
+        <v>SAUNA</v>
+      </c>
+      <c r="G10" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H10" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I10" t="str">
+        <v>CT02</v>
+      </c>
+      <c r="J10" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B11" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ACT020</v>
+      </c>
+      <c r="D11" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="E11" t="str">
+        <v>22</v>
+      </c>
+      <c r="F11" t="str">
+        <v>TURCO</v>
+      </c>
+      <c r="G11" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H11" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Sin asignar</v>
+      </c>
+      <c r="J11" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v>Zona especial sin contratista</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B12" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C12" t="str">
+        <v>ACT030</v>
+      </c>
+      <c r="D12" t="str">
+        <v>CAP04</v>
+      </c>
+      <c r="E12" t="str">
+        <v>6</v>
+      </c>
+      <c r="F12" t="str">
+        <v>601</v>
+      </c>
+      <c r="G12" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H12" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I12" t="str">
+        <v>CT02</v>
+      </c>
+      <c r="J12" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B13" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ACT031</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CAP04</v>
+      </c>
+      <c r="E13" t="str">
+        <v>4</v>
+      </c>
+      <c r="F13" t="str">
+        <v>401</v>
+      </c>
+      <c r="G13" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H13" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I13" t="str">
+        <v>CT02</v>
+      </c>
+      <c r="J13" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B14" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C14" t="str">
+        <v>ACT040</v>
+      </c>
+      <c r="D14" t="str">
+        <v>CAP06</v>
+      </c>
+      <c r="E14" t="str">
+        <v>4</v>
+      </c>
+      <c r="F14" t="str">
+        <v>401</v>
+      </c>
+      <c r="G14" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H14" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I14" t="str">
+        <v>CT03</v>
+      </c>
+      <c r="J14" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K14" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B15" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ACT090</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CAP05</v>
+      </c>
+      <c r="E15" t="str">
+        <v>1</v>
+      </c>
+      <c r="F15" t="str">
+        <v>LOBBY</v>
+      </c>
+      <c r="G15" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H15" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I15" t="str">
+        <v>CT03</v>
+      </c>
+      <c r="J15" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K15" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>P000</v>
+      </c>
+      <c r="B16" t="str">
+        <v>T1</v>
+      </c>
+      <c r="C16" t="str">
+        <v>ACT090</v>
+      </c>
+      <c r="D16" t="str">
+        <v>CAP05</v>
+      </c>
+      <c r="E16" t="str">
+        <v>23</v>
+      </c>
+      <c r="F16" t="str">
+        <v>AMENIDADES</v>
+      </c>
+      <c r="G16" t="str">
+        <v>SI</v>
+      </c>
+      <c r="H16" t="str">
+        <v>SI</v>
+      </c>
+      <c r="I16" t="str">
+        <v>CT03</v>
+      </c>
+      <c r="J16" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K9"/>
   <sheetData>
     <row r="1">
@@ -504,7 +1232,7 @@
         <v>2026-08-18T14:05:00.000Z</v>
       </c>
       <c r="B2" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C2" t="str">
         <v>T1</v>
@@ -531,7 +1259,7 @@
         <v>CT01</v>
       </c>
       <c r="K2" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="3">
@@ -539,7 +1267,7 @@
         <v>2026-08-18T14:06:00.000Z</v>
       </c>
       <c r="B3" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C3" t="str">
         <v>T1</v>
@@ -566,7 +1294,7 @@
         <v>CT01</v>
       </c>
       <c r="K3" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="4">
@@ -574,7 +1302,7 @@
         <v>2026-08-19T09:12:00.000Z</v>
       </c>
       <c r="B4" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C4" t="str">
         <v>T1</v>
@@ -601,7 +1329,7 @@
         <v>CT01</v>
       </c>
       <c r="K4" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="5">
@@ -609,7 +1337,7 @@
         <v>2026-08-19T09:15:00.000Z</v>
       </c>
       <c r="B5" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C5" t="str">
         <v>T1</v>
@@ -636,7 +1364,7 @@
         <v>CT02</v>
       </c>
       <c r="K5" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="6">
@@ -644,7 +1372,7 @@
         <v>2026-08-20T10:30:00.000Z</v>
       </c>
       <c r="B6" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C6" t="str">
         <v>T1</v>
@@ -671,7 +1399,7 @@
         <v>CT02</v>
       </c>
       <c r="K6" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="7">
@@ -679,7 +1407,7 @@
         <v>2026-08-20T10:32:00.000Z</v>
       </c>
       <c r="B7" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C7" t="str">
         <v>T1</v>
@@ -706,7 +1434,7 @@
         <v>CT02</v>
       </c>
       <c r="K7" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="8">
@@ -714,7 +1442,7 @@
         <v>2026-08-21T16:00:00.000Z</v>
       </c>
       <c r="B8" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C8" t="str">
         <v>T1</v>
@@ -741,7 +1469,7 @@
         <v>CT03</v>
       </c>
       <c r="K8" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
     <row r="9">
@@ -749,7 +1477,7 @@
         <v>2026-08-22T08:40:00.000Z</v>
       </c>
       <c r="B9" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="C9" t="str">
         <v>T1</v>
@@ -776,7 +1504,7 @@
         <v>CT02</v>
       </c>
       <c r="K9" t="str">
-        <v>111222333</v>
+        <v>residente@urbanizadorajimenez.com</v>
       </c>
     </row>
   </sheetData>
@@ -803,10 +1531,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P001</v>
+        <v>E001</v>
       </c>
       <c r="B2" t="str">
-        <v>SALGUERO ELITE 2</v>
+        <v>URBANIZADORA JIMENEZ</v>
       </c>
       <c r="C2" t="str">
         <v>SI</v>
@@ -821,250 +1549,354 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ID_USUARIO</v>
+        <v>EMPRESA</v>
       </c>
       <c r="B1" t="str">
+        <v>CODIGO</v>
+      </c>
+      <c r="C1" t="str">
         <v>NOMBRE</v>
       </c>
-      <c r="C1" t="str">
-        <v>ROL</v>
-      </c>
       <c r="D1" t="str">
-        <v>PROYECTO</v>
+        <v>ACTIVO</v>
       </c>
       <c r="E1" t="str">
-        <v>TORRE</v>
-      </c>
-      <c r="F1" t="str">
-        <v>SENDER_ID</v>
-      </c>
-      <c r="G1" t="str">
-        <v>PIN_HASH</v>
-      </c>
-      <c r="H1" t="str">
-        <v>ACTIVO</v>
+        <v>DEMO</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>U001</v>
+        <v>E001</v>
       </c>
       <c r="B2" t="str">
-        <v>Darwin</v>
+        <v>P000</v>
       </c>
       <c r="C2" t="str">
-        <v>ADMIN</v>
+        <v>SALGUERO ELITE 1</v>
       </c>
       <c r="D2" t="str">
-        <v>P001</v>
+        <v>SI</v>
       </c>
       <c r="E2" t="str">
-        <v>*</v>
-      </c>
-      <c r="F2" t="str">
-        <v>999000111</v>
-      </c>
-      <c r="G2" t="str">
-        <v>03ac674216f3e15c761ee1a5e255f067953623c8b388b4459e13f978d7c846f4</v>
-      </c>
-      <c r="H2" t="str">
         <v>SI</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>U002</v>
+        <v>E001</v>
       </c>
       <c r="B3" t="str">
-        <v>Laura</v>
+        <v>P001</v>
       </c>
       <c r="C3" t="str">
-        <v>RESIDENTE</v>
+        <v>SALGUERO ELITE 2</v>
       </c>
       <c r="D3" t="str">
-        <v>P001</v>
+        <v>SI</v>
       </c>
       <c r="E3" t="str">
-        <v>T1</v>
-      </c>
-      <c r="F3" t="str">
-        <v>111222333</v>
-      </c>
-      <c r="G3" t="str">
-        <v>03ac674216f3e15c761ee1a5e255f067953623c8b388b4459e13f978d7c846f4</v>
-      </c>
-      <c r="H3" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>U003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Gerencia</v>
-      </c>
-      <c r="C4" t="str">
-        <v>VISUALIZADOR</v>
-      </c>
-      <c r="D4" t="str">
-        <v>P001</v>
-      </c>
-      <c r="E4" t="str">
-        <v>*</v>
-      </c>
-      <c r="F4" t="str">
-        <v>444555666</v>
-      </c>
-      <c r="G4" t="str">
-        <v>03ac674216f3e15c761ee1a5e255f067953623c8b388b4459e13f978d7c846f4</v>
-      </c>
-      <c r="H4" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:N1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>CODIGO</v>
+        <v>ID_USUARIO</v>
       </c>
       <c r="B1" t="str">
         <v>NOMBRE</v>
       </c>
       <c r="C1" t="str">
+        <v>EMAIL</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ROL</v>
+      </c>
+      <c r="E1" t="str">
+        <v>EMPRESA</v>
+      </c>
+      <c r="F1" t="str">
         <v>PROYECTO</v>
       </c>
-      <c r="D1" t="str">
-        <v>PONDERACION</v>
-      </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
+        <v>TORRE</v>
+      </c>
+      <c r="H1" t="str">
+        <v>SENDER_ID</v>
+      </c>
+      <c r="I1" t="str">
+        <v>PASSWORD_HASH</v>
+      </c>
+      <c r="J1" t="str">
+        <v>MUST_CHANGE_PASSWORD</v>
+      </c>
+      <c r="K1" t="str">
+        <v>ACCESS_CODE_HASH</v>
+      </c>
+      <c r="L1" t="str">
+        <v>RESET_PIN_HASH</v>
+      </c>
+      <c r="M1" t="str">
+        <v>RESET_PIN_EXPIRES</v>
+      </c>
+      <c r="N1" t="str">
         <v>ACTIVO</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CAP01</v>
-      </c>
-      <c r="B2" t="str">
-        <v>ESTRUCTURA</v>
-      </c>
-      <c r="C2" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D2" t="str">
-        <v>0.33</v>
-      </c>
-      <c r="E2" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="B3" t="str">
-        <v>MAMPOSTERIA</v>
-      </c>
-      <c r="C3" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D3" t="str">
-        <v>0.12</v>
-      </c>
-      <c r="E3" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>CAP03</v>
-      </c>
-      <c r="B4" t="str">
-        <v>ACABADOS</v>
-      </c>
-      <c r="C4" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D4" t="str">
-        <v>0.25</v>
-      </c>
-      <c r="E4" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>CAP04</v>
-      </c>
-      <c r="B5" t="str">
-        <v>CARPINTERIA MADERA</v>
-      </c>
-      <c r="C5" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D5" t="str">
-        <v>0.10</v>
-      </c>
-      <c r="E5" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>CAP05</v>
-      </c>
-      <c r="B6" t="str">
-        <v>ASEO</v>
-      </c>
-      <c r="C6" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D6" t="str">
-        <v>0.05</v>
-      </c>
-      <c r="E6" t="str">
-        <v>SI</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>CAP06</v>
-      </c>
-      <c r="B7" t="str">
-        <v>PINTURA</v>
-      </c>
-      <c r="C7" t="str">
-        <v>P001</v>
-      </c>
-      <c r="D7" t="str">
-        <v>0.15</v>
-      </c>
-      <c r="E7" t="str">
-        <v>SI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CODIGO</v>
+      </c>
+      <c r="B1" t="str">
+        <v>NOMBRE</v>
+      </c>
+      <c r="C1" t="str">
+        <v>PROYECTO</v>
+      </c>
+      <c r="D1" t="str">
+        <v>PONDERACION</v>
+      </c>
+      <c r="E1" t="str">
+        <v>ACTIVO</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>CAP01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ESTRUCTURA</v>
+      </c>
+      <c r="C2" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0.33</v>
+      </c>
+      <c r="E2" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>MAMPOSTERIA</v>
+      </c>
+      <c r="C3" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D3" t="str">
+        <v>0.12</v>
+      </c>
+      <c r="E3" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ACABADOS</v>
+      </c>
+      <c r="C4" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D4" t="str">
+        <v>0.25</v>
+      </c>
+      <c r="E4" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>CAP04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>CARPINTERIA MADERA</v>
+      </c>
+      <c r="C5" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D5" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="E5" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>CAP05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ASEO</v>
+      </c>
+      <c r="C6" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D6" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="E6" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>CAP06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>PINTURA</v>
+      </c>
+      <c r="C7" t="str">
+        <v>P000</v>
+      </c>
+      <c r="D7" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="E7" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>CAP01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ESTRUCTURA</v>
+      </c>
+      <c r="C8" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D8" t="str">
+        <v>0.33</v>
+      </c>
+      <c r="E8" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>CAP02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MAMPOSTERIA</v>
+      </c>
+      <c r="C9" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D9" t="str">
+        <v>0.12</v>
+      </c>
+      <c r="E9" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>CAP03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ACABADOS</v>
+      </c>
+      <c r="C10" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D10" t="str">
+        <v>0.25</v>
+      </c>
+      <c r="E10" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>CAP04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>CARPINTERIA MADERA</v>
+      </c>
+      <c r="C11" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0.10</v>
+      </c>
+      <c r="E11" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>CAP05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ASEO</v>
+      </c>
+      <c r="C12" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D12" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="E12" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>CAP06</v>
+      </c>
+      <c r="B13" t="str">
+        <v>PINTURA</v>
+      </c>
+      <c r="C13" t="str">
+        <v>P001</v>
+      </c>
+      <c r="D13" t="str">
+        <v>0.15</v>
+      </c>
+      <c r="E13" t="str">
+        <v>SI</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E15"/>
   <sheetData>
@@ -1330,7 +2162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
   <sheetData>
@@ -1385,7 +2217,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D7"/>
   <sheetData>
@@ -1405,7 +2237,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B2" t="str">
         <v>T1</v>
@@ -1419,7 +2251,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B3" t="str">
         <v>T1</v>
@@ -1433,7 +2265,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B4" t="str">
         <v>T1</v>
@@ -1447,7 +2279,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B5" t="str">
         <v>T1</v>
@@ -1461,7 +2293,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B6" t="str">
         <v>T1</v>
@@ -1475,7 +2307,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B7" t="str">
         <v>T1</v>
@@ -1494,7 +2326,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
   <sheetData>
@@ -1520,7 +2352,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B2" t="str">
         <v>T1</v>
@@ -1540,7 +2372,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B3" t="str">
         <v>T1</v>
@@ -1560,7 +2392,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B4" t="str">
         <v>T1</v>
@@ -1580,7 +2412,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B5" t="str">
         <v>T1</v>
@@ -1600,7 +2432,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B6" t="str">
         <v>T1</v>
@@ -1620,7 +2452,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B7" t="str">
         <v>T1</v>
@@ -1640,7 +2472,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B8" t="str">
         <v>T1</v>
@@ -1660,7 +2492,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B9" t="str">
         <v>T1</v>
@@ -1680,7 +2512,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B10" t="str">
         <v>T1</v>
@@ -1700,7 +2532,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B11" t="str">
         <v>T1</v>
@@ -1720,7 +2552,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B12" t="str">
         <v>T1</v>
@@ -1740,7 +2572,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B13" t="str">
         <v>T1</v>
@@ -1760,7 +2592,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>P001</v>
+        <v>P000</v>
       </c>
       <c r="B14" t="str">
         <v>T1</v>
@@ -1783,671 +2615,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M16"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>PROYECTO</v>
-      </c>
-      <c r="B1" t="str">
-        <v>TORRE</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ACTIVIDAD</v>
-      </c>
-      <c r="D1" t="str">
-        <v>CAPITULO</v>
-      </c>
-      <c r="E1" t="str">
-        <v>NIVEL</v>
-      </c>
-      <c r="F1" t="str">
-        <v>UNIDAD</v>
-      </c>
-      <c r="G1" t="str">
-        <v>APLICA</v>
-      </c>
-      <c r="H1" t="str">
-        <v>ACTIVO</v>
-      </c>
-      <c r="I1" t="str">
-        <v>CONTRATISTA</v>
-      </c>
-      <c r="J1" t="str">
-        <v>HABILITADO</v>
-      </c>
-      <c r="K1" t="str">
-        <v>FECHA_ACTIVACION</v>
-      </c>
-      <c r="L1" t="str">
-        <v>FECHA_DESACTIVACION</v>
-      </c>
-      <c r="M1" t="str">
-        <v>OBSERVACION</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C2" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D2" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E2" t="str">
-        <v>4</v>
-      </c>
-      <c r="F2" t="str">
-        <v>401</v>
-      </c>
-      <c r="G2" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H2" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I2" t="str">
-        <v>CT01</v>
-      </c>
-      <c r="J2" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K2" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B3" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D3" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E3" t="str">
-        <v>4</v>
-      </c>
-      <c r="F3" t="str">
-        <v>402</v>
-      </c>
-      <c r="G3" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H3" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Sin asignar</v>
-      </c>
-      <c r="J3" t="str">
-        <v>NO</v>
-      </c>
-      <c r="K3" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
-        <v>Falta firmar contrato</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B4" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D4" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E4" t="str">
-        <v>4</v>
-      </c>
-      <c r="F4" t="str">
-        <v>403</v>
-      </c>
-      <c r="G4" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H4" t="str">
-        <v>NO</v>
-      </c>
-      <c r="I4" t="str">
-        <v>CT01</v>
-      </c>
-      <c r="J4" t="str">
-        <v>NO</v>
-      </c>
-      <c r="K4" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
-        <v>Pausado por diseno</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B5" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C5" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D5" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E5" t="str">
-        <v>4</v>
-      </c>
-      <c r="F5" t="str">
-        <v>404</v>
-      </c>
-      <c r="G5" t="str">
-        <v>NO</v>
-      </c>
-      <c r="H5" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I5" t="str">
-        <v>CT01</v>
-      </c>
-      <c r="J5" t="str">
-        <v>NO</v>
-      </c>
-      <c r="K5" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v>No aplica: fachada norte</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B6" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D6" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E6" t="str">
-        <v>5</v>
-      </c>
-      <c r="F6" t="str">
-        <v>501</v>
-      </c>
-      <c r="G6" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H6" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I6" t="str">
-        <v>CT01</v>
-      </c>
-      <c r="J6" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K6" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B7" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C7" t="str">
-        <v>ACT010</v>
-      </c>
-      <c r="D7" t="str">
-        <v>CAP02</v>
-      </c>
-      <c r="E7" t="str">
-        <v>5</v>
-      </c>
-      <c r="F7" t="str">
-        <v>502</v>
-      </c>
-      <c r="G7" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H7" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I7" t="str">
-        <v>CT01</v>
-      </c>
-      <c r="J7" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K7" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B8" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ACT020</v>
-      </c>
-      <c r="D8" t="str">
-        <v>CAP03</v>
-      </c>
-      <c r="E8" t="str">
-        <v>4</v>
-      </c>
-      <c r="F8" t="str">
-        <v>401</v>
-      </c>
-      <c r="G8" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H8" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I8" t="str">
-        <v>CT02</v>
-      </c>
-      <c r="J8" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K8" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L8" t="str">
-        <v/>
-      </c>
-      <c r="M8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B9" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C9" t="str">
-        <v>ACT020</v>
-      </c>
-      <c r="D9" t="str">
-        <v>CAP03</v>
-      </c>
-      <c r="E9" t="str">
-        <v>4</v>
-      </c>
-      <c r="F9" t="str">
-        <v>402</v>
-      </c>
-      <c r="G9" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H9" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I9" t="str">
-        <v>CT02</v>
-      </c>
-      <c r="J9" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K9" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L9" t="str">
-        <v/>
-      </c>
-      <c r="M9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B10" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C10" t="str">
-        <v>ACT020</v>
-      </c>
-      <c r="D10" t="str">
-        <v>CAP03</v>
-      </c>
-      <c r="E10" t="str">
-        <v>22</v>
-      </c>
-      <c r="F10" t="str">
-        <v>SAUNA</v>
-      </c>
-      <c r="G10" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H10" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I10" t="str">
-        <v>CT02</v>
-      </c>
-      <c r="J10" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K10" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B11" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C11" t="str">
-        <v>ACT020</v>
-      </c>
-      <c r="D11" t="str">
-        <v>CAP03</v>
-      </c>
-      <c r="E11" t="str">
-        <v>22</v>
-      </c>
-      <c r="F11" t="str">
-        <v>TURCO</v>
-      </c>
-      <c r="G11" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H11" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I11" t="str">
-        <v>Sin asignar</v>
-      </c>
-      <c r="J11" t="str">
-        <v>NO</v>
-      </c>
-      <c r="K11" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L11" t="str">
-        <v/>
-      </c>
-      <c r="M11" t="str">
-        <v>Zona especial sin contratista</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B12" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C12" t="str">
-        <v>ACT030</v>
-      </c>
-      <c r="D12" t="str">
-        <v>CAP04</v>
-      </c>
-      <c r="E12" t="str">
-        <v>6</v>
-      </c>
-      <c r="F12" t="str">
-        <v>601</v>
-      </c>
-      <c r="G12" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H12" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I12" t="str">
-        <v>CT02</v>
-      </c>
-      <c r="J12" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K12" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L12" t="str">
-        <v/>
-      </c>
-      <c r="M12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B13" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C13" t="str">
-        <v>ACT031</v>
-      </c>
-      <c r="D13" t="str">
-        <v>CAP04</v>
-      </c>
-      <c r="E13" t="str">
-        <v>4</v>
-      </c>
-      <c r="F13" t="str">
-        <v>401</v>
-      </c>
-      <c r="G13" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H13" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I13" t="str">
-        <v>CT02</v>
-      </c>
-      <c r="J13" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K13" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L13" t="str">
-        <v/>
-      </c>
-      <c r="M13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B14" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C14" t="str">
-        <v>ACT040</v>
-      </c>
-      <c r="D14" t="str">
-        <v>CAP06</v>
-      </c>
-      <c r="E14" t="str">
-        <v>4</v>
-      </c>
-      <c r="F14" t="str">
-        <v>401</v>
-      </c>
-      <c r="G14" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H14" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I14" t="str">
-        <v>CT03</v>
-      </c>
-      <c r="J14" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K14" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L14" t="str">
-        <v/>
-      </c>
-      <c r="M14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B15" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C15" t="str">
-        <v>ACT090</v>
-      </c>
-      <c r="D15" t="str">
-        <v>CAP05</v>
-      </c>
-      <c r="E15" t="str">
-        <v>1</v>
-      </c>
-      <c r="F15" t="str">
-        <v>LOBBY</v>
-      </c>
-      <c r="G15" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H15" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I15" t="str">
-        <v>CT03</v>
-      </c>
-      <c r="J15" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K15" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L15" t="str">
-        <v/>
-      </c>
-      <c r="M15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>P001</v>
-      </c>
-      <c r="B16" t="str">
-        <v>T1</v>
-      </c>
-      <c r="C16" t="str">
-        <v>ACT090</v>
-      </c>
-      <c r="D16" t="str">
-        <v>CAP05</v>
-      </c>
-      <c r="E16" t="str">
-        <v>23</v>
-      </c>
-      <c r="F16" t="str">
-        <v>AMENIDADES</v>
-      </c>
-      <c r="G16" t="str">
-        <v>SI</v>
-      </c>
-      <c r="H16" t="str">
-        <v>SI</v>
-      </c>
-      <c r="I16" t="str">
-        <v>CT03</v>
-      </c>
-      <c r="J16" t="str">
-        <v>SI</v>
-      </c>
-      <c r="K16" t="str">
-        <v>2026-08-01</v>
-      </c>
-      <c r="L16" t="str">
-        <v/>
-      </c>
-      <c r="M16" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M16"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>